<commit_message>
Added Calculation. Fixed connector part number.
</commit_message>
<xml_diff>
--- a/C64 Keyboard connector PCB/Rev. 0/Excel/C64KB_ConPCB_BOM_v0_0.xlsx
+++ b/C64 Keyboard connector PCB/Rev. 0/Excel/C64KB_ConPCB_BOM_v0_0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Projekte\_Eigene\C64-Projects\C64 Keyboard\C64 Keyboard connector PCB\Rev. 0\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{D9C01C3B-920A-42AD-B8F7-4BCA62589D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F0A936-B37A-4408-93BA-F054BF996882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2904" yWindow="0" windowWidth="27036" windowHeight="14700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stückliste" sheetId="1" r:id="rId1"/>
@@ -116,9 +116,6 @@
     <t>369-1-020 or 2-215079-0</t>
   </si>
   <si>
-    <t>Reichelt MPE 369-1-020 or TE Connectivity 9-215083-0</t>
-  </si>
-  <si>
     <t>20-pin IDC socket with strain relief, 2.54mm</t>
   </si>
   <si>
@@ -126,19 +123,28 @@
   </si>
   <si>
     <t>2 layer, Cu 35µ, HASL, 53.0mm x 15.0mm, 1.6mm FR4</t>
+  </si>
+  <si>
+    <t>Reichelt MPE 371-1-020 or TE Connectivity 9-215083-0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Futura Lt BT"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -592,49 +598,49 @@
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -642,10 +648,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -657,19 +663,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1183,24 +1192,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
     </row>
     <row r="2" spans="1:6" ht="20.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
     </row>
     <row r="3" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1229,7 +1238,7 @@
       <c r="B4" s="3">
         <v>1</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D4" s="10" t="s">
@@ -1238,8 +1247,8 @@
       <c r="E4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="13" t="s">
-        <v>33</v>
+      <c r="F4" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
@@ -1247,7 +1256,7 @@
       <c r="B5" s="3">
         <v>1</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -1256,7 +1265,7 @@
       <c r="E5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="11" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1265,7 +1274,7 @@
       <c r="B6" s="3">
         <v>1</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="10" t="s">
@@ -1274,7 +1283,7 @@
       <c r="E6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="11" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1283,7 +1292,7 @@
       <c r="B7" s="3">
         <v>1</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="10" t="s">
@@ -1292,7 +1301,7 @@
       <c r="E7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1301,7 +1310,7 @@
       <c r="B8" s="3">
         <v>1</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="10" t="s">
@@ -1310,23 +1319,23 @@
       <c r="E8" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
-      <c r="B9" s="13">
+      <c r="B9" s="11">
         <v>1</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="4"/>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="11" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1335,15 +1344,15 @@
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="4"/>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="13" t="s">
-        <v>30</v>
+      <c r="F10" s="14" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="6" customFormat="1" ht="27.6" x14ac:dyDescent="0.3">
@@ -1351,15 +1360,15 @@
       <c r="B11" s="3">
         <v>1</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.3">
@@ -1938,7 +1947,7 @@
   <headerFooter>
     <oddFooter>&amp;L&amp;"Futura Lt BT,Light"&amp;F
 Drafted by Sven Petersen&amp;C&amp;"Futura Lt BT,Light"Page &amp;P of &amp;N&amp;R&amp;"Futura Lt BT,Light"&amp;D &amp;T
-Doc.No.: xxx-5-01-00.0</oddFooter>
+Doc.No.: 224-5-01-00.0</oddFooter>
   </headerFooter>
   <ignoredErrors>
     <ignoredError sqref="A4" calculatedColumn="1"/>

</xml_diff>